<commit_message>
Plot nominal covariates as class-count bars
- plot_indicators accepts covariate_array and max_classes; nominal columns
  are drawn as horizontal class-count bars (hatch/alpha/fill styling from
  targetfeaturesymbols), numeric columns keep histogram/boxplot
- Transformation and standardisation skip non-numeric columns
- Default symbols and none transform/standardise for landcover, landuse,
  biogeo16
- LUCAS 2009 select process files renamed to select_list_/select_save_,
  add plot_covariate.json; updated landscape class Excel tables

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lucas/import_data/utility/landscape/excel/biogeo16.xlsx
+++ b/lucas/import_data/utility/landscape/excel/biogeo16.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="55">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -31,6 +31,9 @@
     <t xml:space="preserve">display_name</t>
   </si>
   <si>
+    <t xml:space="preserve">tag</t>
+  </si>
+  <si>
     <t xml:space="preserve">abstract</t>
   </si>
   <si>
@@ -89,6 +92,9 @@
   </si>
   <si>
     <t xml:space="preserve">Black Sea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">black-sea</t>
   </si>
   <si>
     <t xml:space="preserve">A narrow, distinct coastal strip stretching along the southern and western shores of the Black Sea (found in Bulgaria, Romania, and Turkey).</t>
@@ -265,15 +271,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -400,13 +406,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="15.85"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -422,187 +428,229 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>7</v>
+      <c r="E2" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>11</v>
+      <c r="E3" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>15</v>
+      <c r="E4" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>19</v>
+      <c r="E5" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="2" t="s">
         <v>23</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>27</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>31</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>35</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>39</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>45</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D13" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>49</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>51</v>
+      <c r="E14" s="1" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>